<commit_message>
Add Google Analytics GA4 tracking to all pages (G-GY1DFJFTY4)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NorthBeam_BvA.xlsx
+++ b/NorthBeam_BvA.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/516f17199908f130/桌面/Side Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1116" documentId="11_1FD8B5786060DC902A676B94D9BF1D60DE15AA13" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ADC0903B-7E24-40C5-B2C9-3B8BA15C656F}"/>
+  <xr:revisionPtr revIDLastSave="1197" documentId="11_1FD8B5786060DC902A676B94D9BF1D60DE15AA13" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E0103C15-B6DE-46E4-9081-44AB444E975E}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="674" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="674" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover &amp; Scenario" sheetId="1" r:id="rId1"/>
@@ -56,8 +56,11 @@
     <definedName name="Scenarios">#REF!</definedName>
     <definedName name="Segments">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191028" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -82,6 +85,129 @@
     <t>NorthBeam Analytics, Inc.</t>
   </si>
   <si>
+    <t>Side Project 1 — FY2026 Department Budget vs. Actual Variance Analysis</t>
+  </si>
+  <si>
+    <t>Project Information</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Jin-Tang Shen</t>
+  </si>
+  <si>
+    <t>Date Completed</t>
+  </si>
+  <si>
+    <t>Model Purpose</t>
+  </si>
+  <si>
+    <t>This workbook demonstrates a Budget vs. Actual variance analysis, a core recurring FP&amp;A deliverable. The goal is to show I can build a monthly variance tracker, identify favorable/unfavorable trends, and explain the business drivers behind variances in a way a non-financial stakeholder can follow.</t>
+  </si>
+  <si>
+    <t>Model Legend</t>
+  </si>
+  <si>
+    <t>Format Type</t>
+  </si>
+  <si>
+    <t>Example</t>
+  </si>
+  <si>
+    <t>Meaning / Description</t>
+  </si>
+  <si>
+    <t>Blue Font</t>
+  </si>
+  <si>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>Hardcoded Inputs / Assumptions</t>
+  </si>
+  <si>
+    <t>Black Font</t>
+  </si>
+  <si>
+    <t>Formulas &amp; Calculations</t>
+  </si>
+  <si>
+    <t>Light Green Fill</t>
+  </si>
+  <si>
+    <t>Conditional Fill: under budget</t>
+  </si>
+  <si>
+    <t>Light Red Fill</t>
+  </si>
+  <si>
+    <t>Conditional Fill: over budget</t>
+  </si>
+  <si>
+    <t>Navigation Guide</t>
+  </si>
+  <si>
+    <t>Tab 1 — Cover &amp; Scenario</t>
+  </si>
+  <si>
+    <t>Project background, formatting legend, data disclosure, and a brief description of the variance drivers for each department.</t>
+  </si>
+  <si>
+    <t>Tab 2 — Budget vs Actual</t>
+  </si>
+  <si>
+    <t>Monthly Budget vs. Actual figures for all four departments across FY2026, including variance calculations, status indicators, and key variance commentary.</t>
+  </si>
+  <si>
+    <t>Tab 3 — Dashboard</t>
+  </si>
+  <si>
+    <t>Visual summary of FY2026 results with KPI cards and three charts covering department-level spending, monthly trends, and overall variance breakdown.</t>
+  </si>
+  <si>
+    <t>Data Disclosure</t>
+  </si>
+  <si>
+    <t>NorthBeam Analytics is a fictional company. This workbook was created solely for educational and portfolio purposes. All financial data, assumptions, and business scenarios are fictional and do not represent any real organization.</t>
+  </si>
+  <si>
+    <t>Variance Scenario Descriptions</t>
+  </si>
+  <si>
+    <t>Cost of Revenue (COGS)</t>
+  </si>
+  <si>
+    <t>A mid-year cloud infrastructure price increase (AWS) pushed hosting costs steadily above budget from May onward (unfavorable, growing through the year).</t>
+  </si>
+  <si>
+    <t>Sales &amp; Marketing</t>
+  </si>
+  <si>
+    <t>Consistently overspent due to incremental paid ad spend chasing pipeline targets, a trade-show overrun in August, and an aggressive Q4 push (unfavorable in every month).</t>
+  </si>
+  <si>
+    <t>Research &amp; Development</t>
+  </si>
+  <si>
+    <t>Consistently underspent because planned engineering hires were delayed by slow recruiting; open requisitions stayed unfilled for most of the year (favorable in every month).</t>
+  </si>
+  <si>
+    <t>General &amp; Administrative</t>
+  </si>
+  <si>
+    <t>Tracked close to budget all year except October, when a one-time legal settlement cost drove a large unfavorable spike.</t>
+  </si>
+  <si>
+    <t>FY2026 Monthly Operating Expense: Budget vs. Actual (USD)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>FY2026 Operating Expense Budget ($)</t>
+  </si>
+  <si>
     <t>Department</t>
   </si>
   <si>
@@ -124,117 +250,66 @@
     <t>FY Total</t>
   </si>
   <si>
-    <t>Cost of Revenue (COGS)</t>
-  </si>
-  <si>
-    <t>Sales &amp; Marketing</t>
-  </si>
-  <si>
-    <t>Research &amp; Development</t>
-  </si>
-  <si>
-    <t>General &amp; Administrative</t>
-  </si>
-  <si>
     <t>Total Operating Expense</t>
   </si>
   <si>
+    <t xml:space="preserve"> FY2026 Operating Expense Actual ($)</t>
+  </si>
+  <si>
+    <t>Variance ($)</t>
+  </si>
+  <si>
+    <t>Variance (%)</t>
+  </si>
+  <si>
+    <t>Budget Execution Status (F: Favorable / U: Unfavorable)</t>
+  </si>
+  <si>
+    <t>Key Variance Commentary</t>
+  </si>
+  <si>
     <t>Period</t>
   </si>
   <si>
-    <t>Variance ($)</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Likely Driver</t>
   </si>
   <si>
-    <t>Jin-Tang Shen</t>
-  </si>
-  <si>
-    <t>Model Legend</t>
-  </si>
-  <si>
-    <t>Format Type</t>
-  </si>
-  <si>
-    <t>Example</t>
-  </si>
-  <si>
-    <t>Meaning / Description</t>
-  </si>
-  <si>
-    <t>Blue Font</t>
-  </si>
-  <si>
-    <t>Black Font</t>
-  </si>
-  <si>
-    <t>Light Green Fill</t>
-  </si>
-  <si>
-    <t>Light Red Fill</t>
-  </si>
-  <si>
-    <t>ABC</t>
-  </si>
-  <si>
-    <t>Data Disclosure</t>
-  </si>
-  <si>
-    <t>Project Information</t>
-  </si>
-  <si>
-    <t>Model Purpose</t>
-  </si>
-  <si>
-    <t>Hardcoded Inputs / Assumptions</t>
-  </si>
-  <si>
-    <t>Formulas &amp; Calculations</t>
-  </si>
-  <si>
-    <t>This workbook demonstrates a Budget vs. Actual variance analysis, a core recurring FP&amp;A deliverable. The goal is to show I can build a monthly variance tracker, identify favorable/unfavorable trends, and explain the business drivers behind variances in a way a non-financial stakeholder can follow.</t>
-  </si>
-  <si>
-    <t>Variance Scenario Descriptions</t>
-  </si>
-  <si>
-    <t>Date Completed</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Conditional Fill: under budget</t>
-  </si>
-  <si>
-    <t>Conditional Fill: over budget</t>
-  </si>
-  <si>
-    <t>FY2026 Monthly Operating Expense: Budget vs. Actual (USD)</t>
-  </si>
-  <si>
-    <t>Side Project 1 — FY2026 Department Budget vs. Actual Variance Analysis</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> FY2026 Operating Expense Actual ($)</t>
+    <t>Overspend occurred in every single month. Driver was incremental paid ad spend chasing pipeline targets, compounded by a trade-show overrun and an aggressive Q4 push.</t>
+  </si>
+  <si>
+    <t>Aggressive year-end pipeline push added incremental paid ad spend beyond the planned Q4 ramp.</t>
+  </si>
+  <si>
+    <t>Mid-year cloud infrastructure (AWS) price increase pushed hosting costs steadily above budget from May onward.</t>
+  </si>
+  <si>
+    <t>Driver was delayed engineering hiring, not cost discipline. Several requisitions stayed unfilled all year, which is a product roadmap risk, not a result worth celebrating.</t>
+  </si>
+  <si>
+    <t>One-time legal settlement cost was not in the original budget.</t>
+  </si>
+  <si>
+    <t>Total Budget</t>
   </si>
   <si>
     <t>Total Actual</t>
   </si>
   <si>
-    <t>Total Budget</t>
+    <t>Total Variance</t>
+  </si>
+  <si>
+    <t>FY2026 Budget</t>
   </si>
   <si>
     <t>COGS</t>
   </si>
   <si>
+    <t>FY2026 Actual</t>
+  </si>
+  <si>
     <t>S&amp;M</t>
   </si>
   <si>
@@ -242,78 +317,6 @@
   </si>
   <si>
     <t>G&amp;A</t>
-  </si>
-  <si>
-    <t>FY2026 Budget</t>
-  </si>
-  <si>
-    <t>FY2026 Actual</t>
-  </si>
-  <si>
-    <t>Key Variance Commentary</t>
-  </si>
-  <si>
-    <t>Budget Execution Status (F: Favorable / U: Unfavorable)</t>
-  </si>
-  <si>
-    <t>A mid-year cloud infrastructure price increase (AWS) pushed hosting costs steadily above budget from May onward (unfavorable, growing through the year).</t>
-  </si>
-  <si>
-    <t>Consistently overspent due to incremental paid ad spend chasing pipeline targets, a trade-show overrun in August, and an aggressive Q4 push (unfavorable in every month).</t>
-  </si>
-  <si>
-    <t>Tracked close to budget all year except October, when a one-time legal settlement cost drove a large unfavorable spike.</t>
-  </si>
-  <si>
-    <t>Consistently underspent because planned engineering hires were delayed by slow recruiting; open requisitions stayed unfilled for most of the year (favorable in every month).</t>
-  </si>
-  <si>
-    <t>Driver was delayed engineering hiring, not cost discipline. Several requisitions stayed unfilled all year, which is a product roadmap risk, not a result worth celebrating.</t>
-  </si>
-  <si>
-    <t>One-time legal settlement cost was not in the original budget.</t>
-  </si>
-  <si>
-    <t>Aggressive year-end pipeline push added incremental paid ad spend beyond the planned Q4 ramp.</t>
-  </si>
-  <si>
-    <t>Mid-year cloud infrastructure (AWS) price increase pushed hosting costs steadily above budget from May onward.</t>
-  </si>
-  <si>
-    <t>Overspend occurred in every single month. Driver was incremental paid ad spend chasing pipeline targets, compounded by a trade-show overrun and an aggressive Q4 push.</t>
-  </si>
-  <si>
-    <t>FY2026 Operating Expense Budget ($)</t>
-  </si>
-  <si>
-    <t>Variance (%)</t>
-  </si>
-  <si>
-    <t>NorthBeam Analytics is a fictional company. This workbook was created solely for educational and portfolio purposes. All financial data, assumptions, and business scenarios are fictional and do not represent any real organization.</t>
-  </si>
-  <si>
-    <t>Total Variance</t>
-  </si>
-  <si>
-    <t>Navigation Guide</t>
-  </si>
-  <si>
-    <t>Tab 1 — Cover &amp; Scenario</t>
-  </si>
-  <si>
-    <t>Tab 2 — Budget vs Actual</t>
-  </si>
-  <si>
-    <t>Tab 3 — Dashboard</t>
-  </si>
-  <si>
-    <t>Project background, formatting legend, data disclosure, and a brief description of the variance drivers for each department.</t>
-  </si>
-  <si>
-    <t>Monthly Budget vs. Actual figures for all four departments across FY2026, including variance calculations, status indicators, and key variance commentary.</t>
-  </si>
-  <si>
-    <t>Visual summary of FY2026 results with KPI cards and three charts covering department-level spending, monthly trends, and overall variance breakdown.</t>
   </si>
 </sst>
 </file>
@@ -328,7 +331,7 @@
     <numFmt numFmtId="166" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -483,6 +486,13 @@
       <name val="Cambria"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -540,7 +550,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="43">
     <border>
       <left/>
       <right/>
@@ -1006,6 +1016,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -1013,11 +1053,8 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="16" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1084,7 +1121,6 @@
     <xf numFmtId="165" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1126,11 +1162,23 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="29" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="30" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1194,6 +1242,30 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1206,18 +1278,6 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="167" fontId="21" fillId="8" borderId="36" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1239,9 +1299,6 @@
     <xf numFmtId="167" fontId="21" fillId="8" borderId="32" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1263,24 +1320,23 @@
     <xf numFmtId="0" fontId="20" fillId="8" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="8" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -4292,7 +4348,7 @@
         <xdr:cNvPr id="2" name="Chart 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{89A23ED5-11A1-BB7E-9B3B-7F6A30126A05}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4357,8 +4413,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="162036" y="4634528"/>
-              <a:ext cx="9041804" cy="3763273"/>
+              <a:off x="163941" y="4668818"/>
+              <a:ext cx="8988464" cy="3761368"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -4406,7 +4462,7 @@
         <xdr:cNvPr id="6" name="Chart 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{80B6C600-7660-444D-83F4-072D3100B9E7}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0200-000006000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4424,6 +4480,50 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>158400</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>161879</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>192405</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>162093</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ECC03805-77C4-62F9-4F97-DCDB7DDC3003}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="158400" y="4532173"/>
+          <a:ext cx="9267652" cy="3586096"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -4619,239 +4719,238 @@
   <sheetData>
     <row r="1" spans="2:5" ht="12.6" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:5" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="49" t="s">
-        <v>46</v>
+      <c r="B3" s="46" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="57" t="s">
-        <v>35</v>
-      </c>
-      <c r="C5" s="58"/>
+      <c r="B5" s="59" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="60"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B6" s="50" t="s">
-        <v>42</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>24</v>
+      <c r="B6" s="47" t="s">
+        <v>3</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="50" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="17">
+      <c r="B7" s="47" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="16">
         <v>46198</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
-      <c r="C8" s="8"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="7"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="43" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="44"/>
-      <c r="D9" s="44"/>
+      <c r="B9" s="41" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="42"/>
+      <c r="D9" s="42"/>
     </row>
     <row r="10" spans="2:5" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="66" t="s">
-        <v>39</v>
-      </c>
-      <c r="C10" s="67"/>
-      <c r="D10" s="68"/>
-      <c r="E10" s="37"/>
+      <c r="B10" s="68" t="s">
+        <v>7</v>
+      </c>
+      <c r="C10" s="69"/>
+      <c r="D10" s="70"/>
+      <c r="E10" s="35"/>
     </row>
     <row r="11" spans="2:5" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="69"/>
-      <c r="C11" s="70"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="37"/>
+      <c r="B11" s="71"/>
+      <c r="C11" s="72"/>
+      <c r="D11" s="73"/>
+      <c r="E11" s="35"/>
     </row>
     <row r="12" spans="2:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
+      <c r="B12" s="1"/>
     </row>
     <row r="13" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="59" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="60"/>
-      <c r="D13" s="60"/>
+      <c r="B13" s="61" t="s">
+        <v>8</v>
+      </c>
+      <c r="C13" s="62"/>
+      <c r="D13" s="62"/>
     </row>
     <row r="14" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="13" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>28</v>
+      <c r="B14" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="23" t="s">
-        <v>37</v>
+      <c r="B15" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" s="22" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="23" t="s">
-        <v>38</v>
+      <c r="B16" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="22" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="17" spans="2:5" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="23" t="s">
-        <v>43</v>
+      <c r="B17" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="22" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B18" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C18" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="24" t="s">
-        <v>44</v>
+      <c r="B18" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="19" spans="2:5" ht="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="2:5" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="95" t="s">
-        <v>72</v>
-      </c>
-      <c r="C20" s="96"/>
-      <c r="D20" s="96"/>
+      <c r="B20" s="41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20" s="49"/>
+      <c r="D20" s="49"/>
     </row>
     <row r="21" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="97" t="s">
-        <v>73</v>
-      </c>
-      <c r="C21" s="51" t="s">
-        <v>76</v>
-      </c>
-      <c r="D21" s="52"/>
+      <c r="B21" s="50" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="53" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="54"/>
     </row>
     <row r="22" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="97" t="s">
-        <v>74</v>
-      </c>
-      <c r="C22" s="53" t="s">
-        <v>77</v>
-      </c>
-      <c r="D22" s="54"/>
+      <c r="B22" s="50" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="55" t="s">
+        <v>25</v>
+      </c>
+      <c r="D22" s="56"/>
     </row>
     <row r="23" spans="2:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="98" t="s">
-        <v>75</v>
-      </c>
-      <c r="C23" s="101" t="s">
-        <v>78</v>
-      </c>
-      <c r="D23" s="100"/>
+      <c r="B23" s="51" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="74" t="s">
+        <v>27</v>
+      </c>
+      <c r="D23" s="75"/>
     </row>
     <row r="24" spans="2:5" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C24" s="99"/>
-      <c r="D24" s="99"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B25" s="61" t="s">
+      <c r="B25" s="63" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="64"/>
+      <c r="D25" s="64"/>
+    </row>
+    <row r="26" spans="2:5" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="65" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="66"/>
+      <c r="D26" s="67"/>
+    </row>
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B27" s="1"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="63" t="s">
+        <v>30</v>
+      </c>
+      <c r="C28" s="64"/>
+      <c r="D28" s="64"/>
+    </row>
+    <row r="29" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="33" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="D29" s="54"/>
+    </row>
+    <row r="30" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="33" t="s">
+        <v>33</v>
+      </c>
+      <c r="C30" s="53" t="s">
         <v>34</v>
       </c>
-      <c r="C25" s="62"/>
-      <c r="D25" s="62"/>
-    </row>
-    <row r="26" spans="2:5" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="63" t="s">
-        <v>70</v>
-      </c>
-      <c r="C26" s="64"/>
-      <c r="D26" s="65"/>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B27" s="2"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B28" s="61" t="s">
-        <v>40</v>
-      </c>
-      <c r="C28" s="62"/>
-      <c r="D28" s="62"/>
-    </row>
-    <row r="29" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="35" t="s">
-        <v>15</v>
-      </c>
-      <c r="C29" s="51" t="s">
-        <v>59</v>
-      </c>
-      <c r="D29" s="52"/>
-    </row>
-    <row r="30" spans="2:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="51" t="s">
-        <v>60</v>
-      </c>
-      <c r="D30" s="52"/>
+      <c r="D30" s="54"/>
     </row>
     <row r="31" spans="2:5" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="35" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="53" t="s">
-        <v>62</v>
-      </c>
-      <c r="D31" s="54"/>
+      <c r="B31" s="33" t="s">
+        <v>35</v>
+      </c>
+      <c r="C31" s="55" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" s="56"/>
     </row>
     <row r="32" spans="2:5" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="36" t="s">
-        <v>18</v>
-      </c>
-      <c r="C32" s="55" t="s">
-        <v>61</v>
-      </c>
-      <c r="D32" s="56"/>
-      <c r="E32" s="37"/>
+      <c r="B32" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="57" t="s">
+        <v>38</v>
+      </c>
+      <c r="D32" s="58"/>
+      <c r="E32" s="35"/>
     </row>
     <row r="34" spans="3:4" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D34" s="12"/>
+      <c r="D34" s="11"/>
     </row>
     <row r="35" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="D35" s="12"/>
+      <c r="D35" s="11"/>
     </row>
     <row r="36" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C36" s="12"/>
+      <c r="C36" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="C23:D23"/>
     <mergeCell ref="C29:D29"/>
     <mergeCell ref="C30:D30"/>
     <mergeCell ref="C31:D31"/>
@@ -4864,6 +4963,7 @@
     <mergeCell ref="B10:D11"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C22:D22"/>
+    <mergeCell ref="C23:D23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -4882,1694 +4982,1709 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="80" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="80"/>
+      <c r="C1" s="80"/>
+      <c r="D1" s="80"/>
+      <c r="E1" s="80"/>
+      <c r="F1" s="80"/>
+      <c r="G1" s="80"/>
+      <c r="H1" s="80"/>
+      <c r="I1" s="80"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="48" t="s">
-        <v>45</v>
-      </c>
+      <c r="A2" s="81" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="81"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="O3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" s="59" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" s="82"/>
+      <c r="C4" s="82"/>
+      <c r="D4" s="82"/>
+      <c r="E4" s="82"/>
+      <c r="F4" s="82"/>
+      <c r="G4" s="82"/>
+      <c r="H4" s="82"/>
+      <c r="I4" s="82"/>
+      <c r="J4" s="82"/>
+      <c r="K4" s="82"/>
+      <c r="L4" s="82"/>
+      <c r="M4" s="82"/>
+      <c r="N4" s="83"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C5" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D5" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="F5" s="48" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" s="74" t="s">
-        <v>68</v>
-      </c>
-      <c r="B4" s="75"/>
-      <c r="C4" s="75"/>
-      <c r="D4" s="75"/>
-      <c r="E4" s="75"/>
-      <c r="F4" s="75"/>
-      <c r="G4" s="75"/>
-      <c r="H4" s="75"/>
-      <c r="I4" s="75"/>
-      <c r="J4" s="75"/>
-      <c r="K4" s="75"/>
-      <c r="L4" s="75"/>
-      <c r="M4" s="75"/>
-      <c r="N4" s="58"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M5" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N5" s="1" t="s">
-        <v>14</v>
+      <c r="G5" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="H5" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="I5" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="K5" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="L5" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="M5" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="N5" s="48" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="14">
+      <c r="A6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="13">
         <v>780000</v>
       </c>
-      <c r="C6" s="14">
+      <c r="C6" s="13">
         <v>790000</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="13">
         <v>800000</v>
       </c>
-      <c r="E6" s="14">
+      <c r="E6" s="13">
         <v>810000</v>
       </c>
-      <c r="F6" s="14">
+      <c r="F6" s="13">
         <v>820000</v>
       </c>
-      <c r="G6" s="14">
+      <c r="G6" s="13">
         <v>830000</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="13">
         <v>840000</v>
       </c>
-      <c r="I6" s="14">
+      <c r="I6" s="13">
         <v>850000</v>
       </c>
-      <c r="J6" s="14">
+      <c r="J6" s="13">
         <v>860000</v>
       </c>
-      <c r="K6" s="14">
+      <c r="K6" s="13">
         <v>870000</v>
       </c>
-      <c r="L6" s="14">
+      <c r="L6" s="13">
         <v>880000</v>
       </c>
-      <c r="M6" s="14">
+      <c r="M6" s="13">
         <v>900000</v>
       </c>
-      <c r="N6" s="10">
+      <c r="N6" s="9">
         <f>SUM(B6:M6)</f>
         <v>10030000</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="14">
+      <c r="A7" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" s="13">
         <v>1500000</v>
       </c>
-      <c r="C7" s="14">
+      <c r="C7" s="13">
         <v>1500000</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="13">
         <v>1550000</v>
       </c>
-      <c r="E7" s="14">
+      <c r="E7" s="13">
         <v>1550000</v>
       </c>
-      <c r="F7" s="14">
+      <c r="F7" s="13">
         <v>1600000</v>
       </c>
-      <c r="G7" s="14">
+      <c r="G7" s="13">
         <v>1600000</v>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="13">
         <v>1650000</v>
       </c>
-      <c r="I7" s="14">
+      <c r="I7" s="13">
         <v>1850000</v>
       </c>
-      <c r="J7" s="14">
+      <c r="J7" s="13">
         <v>1650000</v>
       </c>
-      <c r="K7" s="14">
+      <c r="K7" s="13">
         <v>1800000</v>
       </c>
-      <c r="L7" s="14">
+      <c r="L7" s="13">
         <v>1900000</v>
       </c>
-      <c r="M7" s="14">
+      <c r="M7" s="13">
         <v>2200000</v>
       </c>
-      <c r="N7" s="10">
+      <c r="N7" s="9">
         <f t="shared" ref="N7:N9" si="0">SUM(B7:M7)</f>
         <v>20350000</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="14">
+      <c r="A8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="13">
         <v>950000</v>
       </c>
-      <c r="C8" s="14">
+      <c r="C8" s="13">
         <v>950000</v>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="13">
         <v>1000000</v>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="13">
         <v>1000000</v>
       </c>
-      <c r="F8" s="14">
+      <c r="F8" s="13">
         <v>1050000</v>
       </c>
-      <c r="G8" s="14">
+      <c r="G8" s="13">
         <v>1050000</v>
       </c>
-      <c r="H8" s="14">
+      <c r="H8" s="13">
         <v>1100000</v>
       </c>
-      <c r="I8" s="14">
+      <c r="I8" s="13">
         <v>1100000</v>
       </c>
-      <c r="J8" s="14">
+      <c r="J8" s="13">
         <v>1100000</v>
       </c>
-      <c r="K8" s="14">
+      <c r="K8" s="13">
         <v>1100000</v>
       </c>
-      <c r="L8" s="14">
+      <c r="L8" s="13">
         <v>1100000</v>
       </c>
-      <c r="M8" s="14">
+      <c r="M8" s="13">
         <v>1050000</v>
       </c>
-      <c r="N8" s="10">
+      <c r="N8" s="9">
         <f t="shared" si="0"/>
         <v>12550000</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="14">
+      <c r="A9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="13">
         <v>400000</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="13">
         <v>400000</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="13">
         <v>400000</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="13">
         <v>410000</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="13">
         <v>500000</v>
       </c>
-      <c r="G9" s="14">
+      <c r="G9" s="13">
         <v>410000</v>
       </c>
-      <c r="H9" s="14">
+      <c r="H9" s="13">
         <v>410000</v>
       </c>
-      <c r="I9" s="14">
+      <c r="I9" s="13">
         <v>410000</v>
       </c>
-      <c r="J9" s="14">
+      <c r="J9" s="13">
         <v>420000</v>
       </c>
-      <c r="K9" s="14">
+      <c r="K9" s="13">
         <v>420000</v>
       </c>
-      <c r="L9" s="14">
+      <c r="L9" s="13">
         <v>420000</v>
       </c>
-      <c r="M9" s="14">
+      <c r="M9" s="13">
         <v>420000</v>
       </c>
-      <c r="N9" s="10">
+      <c r="N9" s="9">
         <f t="shared" si="0"/>
         <v>5020000</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="10">
+      <c r="A10" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="9">
         <f>SUM(B6:B9)</f>
         <v>3630000</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="9">
         <f t="shared" ref="C10:M10" si="1">SUM(C6:C9)</f>
         <v>3640000</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="9">
         <f t="shared" si="1"/>
         <v>3750000</v>
       </c>
-      <c r="E10" s="10">
+      <c r="E10" s="9">
         <f t="shared" si="1"/>
         <v>3770000</v>
       </c>
-      <c r="F10" s="10">
+      <c r="F10" s="9">
         <f t="shared" si="1"/>
         <v>3970000</v>
       </c>
-      <c r="G10" s="10">
+      <c r="G10" s="9">
         <f t="shared" si="1"/>
         <v>3890000</v>
       </c>
-      <c r="H10" s="10">
+      <c r="H10" s="9">
         <f t="shared" si="1"/>
         <v>4000000</v>
       </c>
-      <c r="I10" s="10">
+      <c r="I10" s="9">
         <f t="shared" si="1"/>
         <v>4210000</v>
       </c>
-      <c r="J10" s="10">
+      <c r="J10" s="9">
         <f t="shared" si="1"/>
         <v>4030000</v>
       </c>
-      <c r="K10" s="10">
+      <c r="K10" s="9">
         <f t="shared" si="1"/>
         <v>4190000</v>
       </c>
-      <c r="L10" s="10">
+      <c r="L10" s="9">
         <f t="shared" si="1"/>
         <v>4300000</v>
       </c>
-      <c r="M10" s="10">
+      <c r="M10" s="9">
         <f t="shared" si="1"/>
         <v>4570000</v>
       </c>
-      <c r="N10" s="10">
+      <c r="N10" s="9">
         <f>SUM(N6:N9)</f>
         <v>47950000</v>
       </c>
-      <c r="O10" s="5"/>
+      <c r="O10" s="4"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="74" t="s">
+      <c r="A12" s="84" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="85"/>
+      <c r="C12" s="85"/>
+      <c r="D12" s="85"/>
+      <c r="E12" s="85"/>
+      <c r="F12" s="85"/>
+      <c r="G12" s="85"/>
+      <c r="H12" s="85"/>
+      <c r="I12" s="85"/>
+      <c r="J12" s="85"/>
+      <c r="K12" s="85"/>
+      <c r="L12" s="85"/>
+      <c r="M12" s="85"/>
+      <c r="N12" s="60"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B13" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C13" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D13" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E13" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="F13" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G13" s="48" t="s">
         <v>48</v>
       </c>
-      <c r="B12" s="75"/>
-      <c r="C12" s="75"/>
-      <c r="D12" s="75"/>
-      <c r="E12" s="75"/>
-      <c r="F12" s="75"/>
-      <c r="G12" s="75"/>
-      <c r="H12" s="75"/>
-      <c r="I12" s="75"/>
-      <c r="J12" s="75"/>
-      <c r="K12" s="75"/>
-      <c r="L12" s="75"/>
-      <c r="M12" s="75"/>
-      <c r="N12" s="58"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I13" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N13" s="1" t="s">
-        <v>14</v>
+      <c r="H13" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="I13" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="J13" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="K13" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="L13" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="M13" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="N13" s="48" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="14">
+      <c r="A14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="13">
         <v>785000</v>
       </c>
-      <c r="C14" s="14">
+      <c r="C14" s="13">
         <v>795000</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="13">
         <v>810000</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="13">
         <v>825000</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="13">
         <v>850000</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="13">
         <v>870000</v>
       </c>
-      <c r="H14" s="14">
+      <c r="H14" s="13">
         <v>890000</v>
       </c>
-      <c r="I14" s="14">
+      <c r="I14" s="13">
         <v>905000</v>
       </c>
-      <c r="J14" s="14">
+      <c r="J14" s="13">
         <v>920000</v>
       </c>
-      <c r="K14" s="14">
+      <c r="K14" s="13">
         <v>930000</v>
       </c>
-      <c r="L14" s="14">
+      <c r="L14" s="13">
         <v>945000</v>
       </c>
-      <c r="M14" s="14">
+      <c r="M14" s="13">
         <v>970000</v>
       </c>
-      <c r="N14" s="10">
+      <c r="N14" s="9">
         <f>SUM(B14:M14)</f>
         <v>10495000</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B15" s="14">
+      <c r="A15" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="13">
         <v>1480000</v>
       </c>
-      <c r="C15" s="14">
+      <c r="C15" s="13">
         <v>1520000</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="13">
         <v>1600000</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="13">
         <v>1580000</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="13">
         <v>1650000</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="13">
         <v>1700000</v>
       </c>
-      <c r="H15" s="14">
+      <c r="H15" s="13">
         <v>1750000</v>
       </c>
-      <c r="I15" s="14">
+      <c r="I15" s="13">
         <v>2100000</v>
       </c>
-      <c r="J15" s="14">
+      <c r="J15" s="13">
         <v>1800000</v>
       </c>
-      <c r="K15" s="14">
+      <c r="K15" s="13">
         <v>2000000</v>
       </c>
-      <c r="L15" s="14">
+      <c r="L15" s="13">
         <v>2050000</v>
       </c>
-      <c r="M15" s="14">
+      <c r="M15" s="13">
         <v>2500000</v>
       </c>
-      <c r="N15" s="10">
+      <c r="N15" s="9">
         <f t="shared" ref="N15:N18" si="2">SUM(B15:M15)</f>
         <v>21730000</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="14">
+      <c r="A16" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B16" s="13">
         <v>900000</v>
       </c>
-      <c r="C16" s="14">
+      <c r="C16" s="13">
         <v>880000</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="13">
         <v>920000</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="13">
         <v>950000</v>
       </c>
-      <c r="F16" s="14">
+      <c r="F16" s="13">
         <v>980000</v>
       </c>
-      <c r="G16" s="14">
+      <c r="G16" s="13">
         <v>1000000</v>
       </c>
-      <c r="H16" s="14">
+      <c r="H16" s="13">
         <v>1020000</v>
       </c>
-      <c r="I16" s="14">
+      <c r="I16" s="13">
         <v>1050000</v>
       </c>
-      <c r="J16" s="14">
+      <c r="J16" s="13">
         <v>1070000</v>
       </c>
-      <c r="K16" s="14">
+      <c r="K16" s="13">
         <v>1080000</v>
       </c>
-      <c r="L16" s="14">
+      <c r="L16" s="13">
         <v>1090000</v>
       </c>
-      <c r="M16" s="14">
+      <c r="M16" s="13">
         <v>1000000</v>
       </c>
-      <c r="N16" s="10">
+      <c r="N16" s="9">
         <f t="shared" si="2"/>
         <v>11940000</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="14">
+      <c r="A17" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B17" s="13">
         <v>395000</v>
       </c>
-      <c r="C17" s="14">
+      <c r="C17" s="13">
         <v>405000</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="13">
         <v>398000</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="13">
         <v>415000</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="13">
         <v>510000</v>
       </c>
-      <c r="G17" s="14">
+      <c r="G17" s="13">
         <v>405000</v>
       </c>
-      <c r="H17" s="14">
+      <c r="H17" s="13">
         <v>415000</v>
       </c>
-      <c r="I17" s="14">
+      <c r="I17" s="13">
         <v>408000</v>
       </c>
-      <c r="J17" s="14">
+      <c r="J17" s="13">
         <v>425000</v>
       </c>
-      <c r="K17" s="14">
+      <c r="K17" s="13">
         <v>580000</v>
       </c>
-      <c r="L17" s="14">
+      <c r="L17" s="13">
         <v>415000</v>
       </c>
-      <c r="M17" s="14">
+      <c r="M17" s="13">
         <v>425000</v>
       </c>
-      <c r="N17" s="10">
+      <c r="N17" s="9">
         <f t="shared" si="2"/>
         <v>5196000</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B18" s="10">
+      <c r="A18" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="9">
         <f>SUM(B14:B17)</f>
         <v>3560000</v>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <f t="shared" ref="C18:M18" si="3">SUM(C14:C17)</f>
         <v>3600000</v>
       </c>
-      <c r="D18" s="10">
+      <c r="D18" s="9">
         <f t="shared" si="3"/>
         <v>3728000</v>
       </c>
-      <c r="E18" s="10">
+      <c r="E18" s="9">
         <f t="shared" si="3"/>
         <v>3770000</v>
       </c>
-      <c r="F18" s="10">
+      <c r="F18" s="9">
         <f t="shared" si="3"/>
         <v>3990000</v>
       </c>
-      <c r="G18" s="10">
+      <c r="G18" s="9">
         <f t="shared" si="3"/>
         <v>3975000</v>
       </c>
-      <c r="H18" s="10">
+      <c r="H18" s="9">
         <f t="shared" si="3"/>
         <v>4075000</v>
       </c>
-      <c r="I18" s="10">
+      <c r="I18" s="9">
         <f t="shared" si="3"/>
         <v>4463000</v>
       </c>
-      <c r="J18" s="10">
+      <c r="J18" s="9">
         <f t="shared" si="3"/>
         <v>4215000</v>
       </c>
-      <c r="K18" s="10">
+      <c r="K18" s="9">
         <f t="shared" si="3"/>
         <v>4590000</v>
       </c>
-      <c r="L18" s="10">
+      <c r="L18" s="9">
         <f t="shared" si="3"/>
         <v>4500000</v>
       </c>
-      <c r="M18" s="10">
+      <c r="M18" s="9">
         <f t="shared" si="3"/>
         <v>4895000</v>
       </c>
-      <c r="N18" s="10">
+      <c r="N18" s="9">
         <f t="shared" si="2"/>
         <v>49361000</v>
       </c>
-      <c r="O18" s="5"/>
+      <c r="O18" s="4"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="B20" s="72"/>
-      <c r="C20" s="72"/>
-      <c r="D20" s="72"/>
-      <c r="E20" s="72"/>
-      <c r="F20" s="72"/>
-      <c r="G20" s="72"/>
-      <c r="H20" s="72"/>
-      <c r="I20" s="72"/>
-      <c r="J20" s="72"/>
-      <c r="K20" s="72"/>
-      <c r="L20" s="72"/>
-      <c r="M20" s="72"/>
-      <c r="N20" s="73"/>
+      <c r="A20" s="59" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="82"/>
+      <c r="C20" s="82"/>
+      <c r="D20" s="82"/>
+      <c r="E20" s="82"/>
+      <c r="F20" s="82"/>
+      <c r="G20" s="82"/>
+      <c r="H20" s="82"/>
+      <c r="I20" s="82"/>
+      <c r="J20" s="82"/>
+      <c r="K20" s="82"/>
+      <c r="L20" s="82"/>
+      <c r="M20" s="82"/>
+      <c r="N20" s="83"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E21" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F21" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I21" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J21" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K21" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M21" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N21" s="1" t="s">
-        <v>14</v>
+      <c r="A21" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D21" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E21" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="F21" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G21" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="H21" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="I21" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="J21" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="K21" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="L21" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="M21" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="N21" s="48" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B22" s="6">
+      <c r="A22" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B22" s="5">
         <f>B14-B6</f>
         <v>5000</v>
       </c>
-      <c r="C22" s="6">
+      <c r="C22" s="5">
         <f t="shared" ref="C22:M22" si="4">C14-C6</f>
         <v>5000</v>
       </c>
-      <c r="D22" s="6">
+      <c r="D22" s="5">
         <f t="shared" si="4"/>
         <v>10000</v>
       </c>
-      <c r="E22" s="6">
+      <c r="E22" s="5">
         <f t="shared" si="4"/>
         <v>15000</v>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="5">
         <f t="shared" si="4"/>
         <v>30000</v>
       </c>
-      <c r="G22" s="6">
+      <c r="G22" s="5">
         <f t="shared" si="4"/>
         <v>40000</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="5">
         <f t="shared" si="4"/>
         <v>50000</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="5">
         <f t="shared" si="4"/>
         <v>55000</v>
       </c>
-      <c r="J22" s="6">
+      <c r="J22" s="5">
         <f t="shared" si="4"/>
         <v>60000</v>
       </c>
-      <c r="K22" s="6">
+      <c r="K22" s="5">
         <f t="shared" si="4"/>
         <v>60000</v>
       </c>
-      <c r="L22" s="6">
+      <c r="L22" s="5">
         <f t="shared" si="4"/>
         <v>65000</v>
       </c>
-      <c r="M22" s="6">
+      <c r="M22" s="5">
         <f t="shared" si="4"/>
         <v>70000</v>
       </c>
-      <c r="N22" s="10">
+      <c r="N22" s="9">
         <f>SUM(B22:M22)</f>
         <v>465000</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="32" t="s">
-        <v>16</v>
-      </c>
-      <c r="B23" s="6">
+      <c r="A23" s="30" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="5">
         <f t="shared" ref="B23:M23" si="5">B15-B7</f>
         <v>-20000</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="5">
         <f t="shared" si="5"/>
         <v>20000</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="5">
         <f t="shared" si="5"/>
         <v>50000</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="5">
         <f t="shared" si="5"/>
         <v>30000</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="5">
         <f t="shared" si="5"/>
         <v>50000</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="5">
         <f t="shared" si="5"/>
         <v>100000</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="5">
         <f t="shared" si="5"/>
         <v>100000</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="5">
         <f t="shared" si="5"/>
         <v>250000</v>
       </c>
-      <c r="J23" s="6">
+      <c r="J23" s="5">
         <f t="shared" si="5"/>
         <v>150000</v>
       </c>
-      <c r="K23" s="6">
+      <c r="K23" s="5">
         <f t="shared" si="5"/>
         <v>200000</v>
       </c>
-      <c r="L23" s="6">
+      <c r="L23" s="5">
         <f t="shared" si="5"/>
         <v>150000</v>
       </c>
-      <c r="M23" s="6">
+      <c r="M23" s="5">
         <f t="shared" si="5"/>
         <v>300000</v>
       </c>
-      <c r="N23" s="10">
+      <c r="N23" s="9">
         <f t="shared" ref="N23:N26" si="6">SUM(B23:M23)</f>
         <v>1380000</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B24" s="6">
+      <c r="A24" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B24" s="5">
         <f t="shared" ref="B24:M24" si="7">B16-B8</f>
         <v>-50000</v>
       </c>
-      <c r="C24" s="6">
+      <c r="C24" s="5">
         <f t="shared" si="7"/>
         <v>-70000</v>
       </c>
-      <c r="D24" s="6">
+      <c r="D24" s="5">
         <f t="shared" si="7"/>
         <v>-80000</v>
       </c>
-      <c r="E24" s="6">
+      <c r="E24" s="5">
         <f t="shared" si="7"/>
         <v>-50000</v>
       </c>
-      <c r="F24" s="6">
+      <c r="F24" s="5">
         <f t="shared" si="7"/>
         <v>-70000</v>
       </c>
-      <c r="G24" s="6">
+      <c r="G24" s="5">
         <f t="shared" si="7"/>
         <v>-50000</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="5">
         <f t="shared" si="7"/>
         <v>-80000</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="5">
         <f t="shared" si="7"/>
         <v>-50000</v>
       </c>
-      <c r="J24" s="6">
+      <c r="J24" s="5">
         <f t="shared" si="7"/>
         <v>-30000</v>
       </c>
-      <c r="K24" s="6">
+      <c r="K24" s="5">
         <f t="shared" si="7"/>
         <v>-20000</v>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="5">
         <f t="shared" si="7"/>
         <v>-10000</v>
       </c>
-      <c r="M24" s="6">
+      <c r="M24" s="5">
         <f t="shared" si="7"/>
         <v>-50000</v>
       </c>
-      <c r="N24" s="10">
+      <c r="N24" s="9">
         <f t="shared" si="6"/>
         <v>-610000</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B25" s="6">
+      <c r="A25" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B25" s="5">
         <f t="shared" ref="B25:M25" si="8">B17-B9</f>
         <v>-5000</v>
       </c>
-      <c r="C25" s="6">
+      <c r="C25" s="5">
         <f t="shared" si="8"/>
         <v>5000</v>
       </c>
-      <c r="D25" s="6">
+      <c r="D25" s="5">
         <f t="shared" si="8"/>
         <v>-2000</v>
       </c>
-      <c r="E25" s="6">
+      <c r="E25" s="5">
         <f t="shared" si="8"/>
         <v>5000</v>
       </c>
-      <c r="F25" s="6">
+      <c r="F25" s="5">
         <f t="shared" si="8"/>
         <v>10000</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="5">
         <f t="shared" si="8"/>
         <v>-5000</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="5">
         <f t="shared" si="8"/>
         <v>5000</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="5">
         <f t="shared" si="8"/>
         <v>-2000</v>
       </c>
-      <c r="J25" s="6">
+      <c r="J25" s="5">
         <f t="shared" si="8"/>
         <v>5000</v>
       </c>
-      <c r="K25" s="6">
+      <c r="K25" s="5">
         <f t="shared" si="8"/>
         <v>160000</v>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="5">
         <f t="shared" si="8"/>
         <v>-5000</v>
       </c>
-      <c r="M25" s="6">
+      <c r="M25" s="5">
         <f t="shared" si="8"/>
         <v>5000</v>
       </c>
-      <c r="N25" s="10">
+      <c r="N25" s="9">
         <f t="shared" si="6"/>
         <v>176000</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B26" s="10">
+      <c r="A26" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B26" s="9">
         <f>SUM(B22:B25)</f>
         <v>-70000</v>
       </c>
-      <c r="C26" s="10">
+      <c r="C26" s="9">
         <f t="shared" ref="C26:M26" si="9">SUM(C22:C25)</f>
         <v>-40000</v>
       </c>
-      <c r="D26" s="10">
+      <c r="D26" s="9">
         <f t="shared" si="9"/>
         <v>-22000</v>
       </c>
-      <c r="E26" s="10">
+      <c r="E26" s="9">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="F26" s="10">
+      <c r="F26" s="9">
         <f t="shared" si="9"/>
         <v>20000</v>
       </c>
-      <c r="G26" s="10">
+      <c r="G26" s="9">
         <f t="shared" si="9"/>
         <v>85000</v>
       </c>
-      <c r="H26" s="10">
+      <c r="H26" s="9">
         <f t="shared" si="9"/>
         <v>75000</v>
       </c>
-      <c r="I26" s="10">
+      <c r="I26" s="9">
         <f t="shared" si="9"/>
         <v>253000</v>
       </c>
-      <c r="J26" s="10">
+      <c r="J26" s="9">
         <f t="shared" si="9"/>
         <v>185000</v>
       </c>
-      <c r="K26" s="10">
+      <c r="K26" s="9">
         <f t="shared" si="9"/>
         <v>400000</v>
       </c>
-      <c r="L26" s="10">
+      <c r="L26" s="9">
         <f t="shared" si="9"/>
         <v>200000</v>
       </c>
-      <c r="M26" s="10">
+      <c r="M26" s="9">
         <f t="shared" si="9"/>
         <v>325000</v>
       </c>
-      <c r="N26" s="10">
+      <c r="N26" s="9">
         <f t="shared" si="6"/>
         <v>1411000</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="57" t="s">
-        <v>69</v>
-      </c>
-      <c r="B28" s="72"/>
-      <c r="C28" s="72"/>
-      <c r="D28" s="72"/>
-      <c r="E28" s="72"/>
-      <c r="F28" s="72"/>
-      <c r="G28" s="72"/>
-      <c r="H28" s="72"/>
-      <c r="I28" s="72"/>
-      <c r="J28" s="72"/>
-      <c r="K28" s="72"/>
-      <c r="L28" s="72"/>
-      <c r="M28" s="72"/>
-      <c r="N28" s="73"/>
+      <c r="A28" s="59" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="82"/>
+      <c r="C28" s="82"/>
+      <c r="D28" s="82"/>
+      <c r="E28" s="82"/>
+      <c r="F28" s="82"/>
+      <c r="G28" s="82"/>
+      <c r="H28" s="82"/>
+      <c r="I28" s="82"/>
+      <c r="J28" s="82"/>
+      <c r="K28" s="82"/>
+      <c r="L28" s="82"/>
+      <c r="M28" s="82"/>
+      <c r="N28" s="83"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D29" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E29" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I29" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J29" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L29" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M29" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N29" s="1" t="s">
-        <v>14</v>
+      <c r="A29" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D29" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="F29" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G29" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="H29" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="I29" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="J29" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="K29" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="L29" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="M29" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="N29" s="48" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="11">
+      <c r="A30" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B30" s="10">
         <f>IFERROR(B22/B6, "-")</f>
         <v>6.41025641025641E-3</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="10">
         <f t="shared" ref="C30:N30" si="10">IFERROR(C22/C6, "-")</f>
         <v>6.3291139240506328E-3</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="10">
         <f t="shared" si="10"/>
         <v>1.2500000000000001E-2</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="10">
         <f t="shared" si="10"/>
         <v>1.8518518518518517E-2</v>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="10">
         <f t="shared" si="10"/>
         <v>3.6585365853658534E-2</v>
       </c>
-      <c r="G30" s="11">
+      <c r="G30" s="10">
         <f t="shared" si="10"/>
         <v>4.8192771084337352E-2</v>
       </c>
-      <c r="H30" s="11">
+      <c r="H30" s="10">
         <f t="shared" si="10"/>
         <v>5.9523809523809521E-2</v>
       </c>
-      <c r="I30" s="11">
+      <c r="I30" s="10">
         <f t="shared" si="10"/>
         <v>6.4705882352941183E-2</v>
       </c>
-      <c r="J30" s="11">
+      <c r="J30" s="10">
         <f t="shared" si="10"/>
         <v>6.9767441860465115E-2</v>
       </c>
-      <c r="K30" s="11">
+      <c r="K30" s="10">
         <f t="shared" si="10"/>
         <v>6.8965517241379309E-2</v>
       </c>
-      <c r="L30" s="11">
+      <c r="L30" s="10">
         <f t="shared" si="10"/>
         <v>7.3863636363636367E-2</v>
       </c>
-      <c r="M30" s="11">
+      <c r="M30" s="10">
         <f t="shared" si="10"/>
         <v>7.7777777777777779E-2</v>
       </c>
-      <c r="N30" s="27">
+      <c r="N30" s="26">
         <f t="shared" si="10"/>
         <v>4.6360917248255237E-2</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B31" s="11">
+      <c r="A31" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="10">
         <f t="shared" ref="B31:N34" si="11">IFERROR(B23/B7, "-")</f>
         <v>-1.3333333333333334E-2</v>
       </c>
-      <c r="C31" s="11">
+      <c r="C31" s="10">
         <f t="shared" si="11"/>
         <v>1.3333333333333334E-2</v>
       </c>
-      <c r="D31" s="11">
+      <c r="D31" s="10">
         <f t="shared" si="11"/>
         <v>3.2258064516129031E-2</v>
       </c>
-      <c r="E31" s="11">
+      <c r="E31" s="10">
         <f t="shared" si="11"/>
         <v>1.935483870967742E-2</v>
       </c>
-      <c r="F31" s="11">
+      <c r="F31" s="10">
         <f t="shared" si="11"/>
         <v>3.125E-2</v>
       </c>
-      <c r="G31" s="11">
+      <c r="G31" s="10">
         <f t="shared" si="11"/>
         <v>6.25E-2</v>
       </c>
-      <c r="H31" s="11">
+      <c r="H31" s="10">
         <f t="shared" si="11"/>
         <v>6.0606060606060608E-2</v>
       </c>
-      <c r="I31" s="11">
+      <c r="I31" s="10">
         <f t="shared" si="11"/>
         <v>0.13513513513513514</v>
       </c>
-      <c r="J31" s="11">
+      <c r="J31" s="10">
         <f t="shared" si="11"/>
         <v>9.0909090909090912E-2</v>
       </c>
-      <c r="K31" s="11">
+      <c r="K31" s="10">
         <f t="shared" si="11"/>
         <v>0.1111111111111111</v>
       </c>
-      <c r="L31" s="11">
+      <c r="L31" s="10">
         <f t="shared" si="11"/>
         <v>7.8947368421052627E-2</v>
       </c>
-      <c r="M31" s="11">
+      <c r="M31" s="10">
         <f t="shared" si="11"/>
         <v>0.13636363636363635</v>
       </c>
-      <c r="N31" s="27">
+      <c r="N31" s="26">
         <f t="shared" ref="N31" si="12">IFERROR(N23/N7, "-")</f>
         <v>6.7813267813267811E-2</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B32" s="11">
+      <c r="A32" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B32" s="10">
         <f t="shared" si="11"/>
         <v>-5.2631578947368418E-2</v>
       </c>
-      <c r="C32" s="11">
+      <c r="C32" s="10">
         <f t="shared" si="11"/>
         <v>-7.3684210526315783E-2</v>
       </c>
-      <c r="D32" s="11">
+      <c r="D32" s="10">
         <f t="shared" si="11"/>
         <v>-0.08</v>
       </c>
-      <c r="E32" s="11">
+      <c r="E32" s="10">
         <f t="shared" si="11"/>
         <v>-0.05</v>
       </c>
-      <c r="F32" s="11">
+      <c r="F32" s="10">
         <f t="shared" si="11"/>
         <v>-6.6666666666666666E-2</v>
       </c>
-      <c r="G32" s="11">
+      <c r="G32" s="10">
         <f t="shared" si="11"/>
         <v>-4.7619047619047616E-2</v>
       </c>
-      <c r="H32" s="11">
+      <c r="H32" s="10">
         <f t="shared" si="11"/>
         <v>-7.2727272727272724E-2</v>
       </c>
-      <c r="I32" s="11">
+      <c r="I32" s="10">
         <f t="shared" si="11"/>
         <v>-4.5454545454545456E-2</v>
       </c>
-      <c r="J32" s="11">
+      <c r="J32" s="10">
         <f t="shared" si="11"/>
         <v>-2.7272727272727271E-2</v>
       </c>
-      <c r="K32" s="11">
+      <c r="K32" s="10">
         <f t="shared" si="11"/>
         <v>-1.8181818181818181E-2</v>
       </c>
-      <c r="L32" s="11">
+      <c r="L32" s="10">
         <f t="shared" si="11"/>
         <v>-9.0909090909090905E-3</v>
       </c>
-      <c r="M32" s="11">
+      <c r="M32" s="10">
         <f t="shared" si="11"/>
         <v>-4.7619047619047616E-2</v>
       </c>
-      <c r="N32" s="27">
+      <c r="N32" s="26">
         <f t="shared" ref="N32" si="13">IFERROR(N24/N8, "-")</f>
         <v>-4.8605577689243028E-2</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B33" s="11">
+      <c r="A33" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B33" s="10">
         <f t="shared" si="11"/>
         <v>-1.2500000000000001E-2</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="10">
         <f t="shared" si="11"/>
         <v>1.2500000000000001E-2</v>
       </c>
-      <c r="D33" s="11">
+      <c r="D33" s="10">
         <f t="shared" si="11"/>
         <v>-5.0000000000000001E-3</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="10">
         <f t="shared" si="11"/>
         <v>1.2195121951219513E-2</v>
       </c>
-      <c r="F33" s="11">
+      <c r="F33" s="10">
         <f t="shared" si="11"/>
         <v>0.02</v>
       </c>
-      <c r="G33" s="11">
+      <c r="G33" s="10">
         <f t="shared" si="11"/>
         <v>-1.2195121951219513E-2</v>
       </c>
-      <c r="H33" s="11">
+      <c r="H33" s="10">
         <f t="shared" si="11"/>
         <v>1.2195121951219513E-2</v>
       </c>
-      <c r="I33" s="11">
+      <c r="I33" s="10">
         <f t="shared" si="11"/>
         <v>-4.8780487804878049E-3</v>
       </c>
-      <c r="J33" s="11">
+      <c r="J33" s="10">
         <f t="shared" si="11"/>
         <v>1.1904761904761904E-2</v>
       </c>
-      <c r="K33" s="11">
+      <c r="K33" s="10">
         <f t="shared" si="11"/>
         <v>0.38095238095238093</v>
       </c>
-      <c r="L33" s="11">
+      <c r="L33" s="10">
         <f t="shared" si="11"/>
         <v>-1.1904761904761904E-2</v>
       </c>
-      <c r="M33" s="11">
+      <c r="M33" s="10">
         <f t="shared" si="11"/>
         <v>1.1904761904761904E-2</v>
       </c>
-      <c r="N33" s="27">
+      <c r="N33" s="26">
         <f t="shared" ref="N33" si="14">IFERROR(N25/N9, "-")</f>
         <v>3.5059760956175301E-2</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A34" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B34" s="27">
+      <c r="A34" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="26">
         <f t="shared" si="11"/>
         <v>-1.928374655647383E-2</v>
       </c>
-      <c r="C34" s="27">
+      <c r="C34" s="26">
         <f t="shared" si="11"/>
         <v>-1.098901098901099E-2</v>
       </c>
-      <c r="D34" s="27">
+      <c r="D34" s="26">
         <f t="shared" si="11"/>
         <v>-5.8666666666666667E-3</v>
       </c>
-      <c r="E34" s="27">
+      <c r="E34" s="26">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="F34" s="27">
+      <c r="F34" s="26">
         <f t="shared" si="11"/>
         <v>5.0377833753148613E-3</v>
       </c>
-      <c r="G34" s="27">
+      <c r="G34" s="26">
         <f t="shared" si="11"/>
         <v>2.1850899742930592E-2</v>
       </c>
-      <c r="H34" s="27">
+      <c r="H34" s="26">
         <f t="shared" si="11"/>
         <v>1.8749999999999999E-2</v>
       </c>
-      <c r="I34" s="27">
+      <c r="I34" s="26">
         <f t="shared" si="11"/>
         <v>6.0095011876484562E-2</v>
       </c>
-      <c r="J34" s="27">
+      <c r="J34" s="26">
         <f t="shared" si="11"/>
         <v>4.590570719602978E-2</v>
       </c>
-      <c r="K34" s="27">
+      <c r="K34" s="26">
         <f t="shared" si="11"/>
         <v>9.5465393794749401E-2</v>
       </c>
-      <c r="L34" s="27">
+      <c r="L34" s="26">
         <f t="shared" si="11"/>
         <v>4.6511627906976744E-2</v>
       </c>
-      <c r="M34" s="27">
+      <c r="M34" s="26">
         <f t="shared" si="11"/>
         <v>7.1115973741794306E-2</v>
       </c>
-      <c r="N34" s="27">
+      <c r="N34" s="26">
         <f t="shared" si="11"/>
         <v>2.9426485922836289E-2</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A36" s="57" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="72"/>
-      <c r="C36" s="72"/>
-      <c r="D36" s="72"/>
-      <c r="E36" s="72"/>
-      <c r="F36" s="72"/>
-      <c r="G36" s="72"/>
-      <c r="H36" s="72"/>
-      <c r="I36" s="72"/>
-      <c r="J36" s="72"/>
-      <c r="K36" s="72"/>
-      <c r="L36" s="72"/>
-      <c r="M36" s="72"/>
-      <c r="N36" s="73"/>
+      <c r="A36" s="59" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="82"/>
+      <c r="C36" s="82"/>
+      <c r="D36" s="82"/>
+      <c r="E36" s="82"/>
+      <c r="F36" s="82"/>
+      <c r="G36" s="82"/>
+      <c r="H36" s="82"/>
+      <c r="I36" s="82"/>
+      <c r="J36" s="82"/>
+      <c r="K36" s="82"/>
+      <c r="L36" s="82"/>
+      <c r="M36" s="82"/>
+      <c r="N36" s="83"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="I37" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="K37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L37" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M37" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N37" s="1" t="s">
-        <v>14</v>
+      <c r="A37" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B37" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="C37" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D37" s="48" t="s">
+        <v>45</v>
+      </c>
+      <c r="E37" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="F37" s="48" t="s">
+        <v>47</v>
+      </c>
+      <c r="G37" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="H37" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="I37" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="J37" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="K37" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="L37" s="48" t="s">
+        <v>53</v>
+      </c>
+      <c r="M37" s="48" t="s">
+        <v>54</v>
+      </c>
+      <c r="N37" s="48" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A38" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B38" s="25" t="str">
+      <c r="A38" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B38" s="24" t="str">
         <f>IF(B6&gt;=B14, "F", "U")</f>
         <v>U</v>
       </c>
-      <c r="C38" s="25" t="str">
+      <c r="C38" s="24" t="str">
         <f>IF(C6&gt;=C14, "F", "U")</f>
         <v>U</v>
       </c>
-      <c r="D38" s="25" t="str">
+      <c r="D38" s="24" t="str">
         <f t="shared" ref="D38:N38" si="15">IF(D6&gt;=D14, "F", "U")</f>
         <v>U</v>
       </c>
-      <c r="E38" s="25" t="str">
+      <c r="E38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="F38" s="25" t="str">
+      <c r="F38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="G38" s="25" t="str">
+      <c r="G38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="H38" s="25" t="str">
+      <c r="H38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="I38" s="25" t="str">
+      <c r="I38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="J38" s="25" t="str">
+      <c r="J38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="K38" s="25" t="str">
+      <c r="K38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="L38" s="25" t="str">
+      <c r="L38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="M38" s="25" t="str">
+      <c r="M38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
-      <c r="N38" s="25" t="str">
+      <c r="N38" s="24" t="str">
         <f t="shared" si="15"/>
         <v>U</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A39" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B39" s="25" t="str">
+      <c r="A39" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="24" t="str">
         <f t="shared" ref="B39:N39" si="16">IF(B7&gt;=B15, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="C39" s="25" t="str">
+      <c r="C39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="D39" s="25" t="str">
+      <c r="D39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="E39" s="25" t="str">
+      <c r="E39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="F39" s="25" t="str">
+      <c r="F39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="G39" s="25" t="str">
+      <c r="G39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="H39" s="25" t="str">
+      <c r="H39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="I39" s="25" t="str">
+      <c r="I39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="J39" s="25" t="str">
+      <c r="J39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="K39" s="25" t="str">
+      <c r="K39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="L39" s="25" t="str">
+      <c r="L39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="M39" s="25" t="str">
+      <c r="M39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
-      <c r="N39" s="25" t="str">
+      <c r="N39" s="24" t="str">
         <f t="shared" si="16"/>
         <v>U</v>
       </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A40" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B40" s="25" t="str">
+      <c r="A40" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B40" s="24" t="str">
         <f t="shared" ref="B40:N40" si="17">IF(B8&gt;=B16, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="C40" s="25" t="str">
+      <c r="C40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="D40" s="25" t="str">
+      <c r="D40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="E40" s="25" t="str">
+      <c r="E40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="F40" s="25" t="str">
+      <c r="F40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="G40" s="25" t="str">
+      <c r="G40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="H40" s="25" t="str">
+      <c r="H40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="I40" s="25" t="str">
+      <c r="I40" s="24" t="str">
         <f>IF(I8&gt;=I16, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="J40" s="25" t="str">
+      <c r="J40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="K40" s="25" t="str">
+      <c r="K40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="L40" s="25" t="str">
+      <c r="L40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="M40" s="25" t="str">
+      <c r="M40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
-      <c r="N40" s="25" t="str">
+      <c r="N40" s="24" t="str">
         <f t="shared" si="17"/>
         <v>F</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="25" t="str">
+      <c r="A41" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B41" s="24" t="str">
         <f>IF(B9&gt;=B17, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="C41" s="25" t="str">
+      <c r="C41" s="24" t="str">
         <f t="shared" ref="C41:N41" si="18">IF(C9&gt;=C17, "F", "U")</f>
         <v>U</v>
       </c>
-      <c r="D41" s="25" t="str">
+      <c r="D41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>F</v>
       </c>
-      <c r="E41" s="25" t="str">
+      <c r="E41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>U</v>
       </c>
-      <c r="F41" s="25" t="str">
+      <c r="F41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>U</v>
       </c>
-      <c r="G41" s="25" t="str">
+      <c r="G41" s="24" t="str">
         <f>IF(G9&gt;=G17, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="H41" s="25" t="str">
+      <c r="H41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>U</v>
       </c>
-      <c r="I41" s="25" t="str">
+      <c r="I41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>F</v>
       </c>
-      <c r="J41" s="25" t="str">
+      <c r="J41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>U</v>
       </c>
-      <c r="K41" s="25" t="str">
+      <c r="K41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>U</v>
       </c>
-      <c r="L41" s="25" t="str">
+      <c r="L41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>F</v>
       </c>
-      <c r="M41" s="25" t="str">
+      <c r="M41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>U</v>
       </c>
-      <c r="N41" s="25" t="str">
+      <c r="N41" s="24" t="str">
         <f t="shared" si="18"/>
         <v>U</v>
       </c>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A42" s="26" t="s">
-        <v>19</v>
-      </c>
-      <c r="B42" s="25" t="str">
+      <c r="A42" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" s="24" t="str">
         <f>IF(B10&gt;=B18, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="C42" s="25" t="str">
+      <c r="C42" s="24" t="str">
         <f>IF(C10&gt;=C18, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="D42" s="25" t="str">
+      <c r="D42" s="24" t="str">
         <f>IF(D10&gt;=D18, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="E42" s="25" t="str">
+      <c r="E42" s="24" t="str">
         <f t="shared" ref="E42:N42" si="19">IF(E10&gt;=E18, "F", "U")</f>
         <v>F</v>
       </c>
-      <c r="F42" s="25" t="str">
+      <c r="F42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="G42" s="25" t="str">
+      <c r="G42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="H42" s="25" t="str">
+      <c r="H42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="I42" s="25" t="str">
+      <c r="I42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="J42" s="25" t="str">
+      <c r="J42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="K42" s="25" t="str">
+      <c r="K42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="L42" s="25" t="str">
+      <c r="L42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="M42" s="25" t="str">
+      <c r="M42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
-      <c r="N42" s="25" t="str">
+      <c r="N42" s="24" t="str">
         <f t="shared" si="19"/>
         <v>U</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A44" s="57" t="s">
-        <v>57</v>
-      </c>
-      <c r="B44" s="72"/>
-      <c r="C44" s="72"/>
-      <c r="D44" s="72"/>
-      <c r="E44" s="72"/>
-      <c r="F44" s="72"/>
-      <c r="G44" s="72"/>
-      <c r="H44" s="72"/>
-      <c r="I44" s="72"/>
-      <c r="J44" s="72"/>
-      <c r="K44" s="72"/>
-      <c r="L44" s="72"/>
-      <c r="M44" s="72"/>
-      <c r="N44" s="73"/>
+      <c r="A44" s="59" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" s="82"/>
+      <c r="C44" s="82"/>
+      <c r="D44" s="82"/>
+      <c r="E44" s="82"/>
+      <c r="F44" s="82"/>
+      <c r="G44" s="82"/>
+      <c r="H44" s="82"/>
+      <c r="I44" s="82"/>
+      <c r="J44" s="82"/>
+      <c r="K44" s="82"/>
+      <c r="L44" s="82"/>
+      <c r="M44" s="82"/>
+      <c r="N44" s="83"/>
     </row>
     <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>22</v>
+      <c r="A45" s="48" t="s">
+        <v>42</v>
+      </c>
+      <c r="B45" s="48" t="s">
+        <v>62</v>
+      </c>
+      <c r="C45" s="48" t="s">
+        <v>58</v>
+      </c>
+      <c r="D45" s="48" t="s">
+        <v>63</v>
       </c>
       <c r="E45" s="79" t="s">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="F45" s="79"/>
       <c r="G45" s="79"/>
@@ -6582,22 +6697,22 @@
       <c r="N45" s="79"/>
     </row>
     <row r="46" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="B46" s="42" t="s">
-        <v>14</v>
-      </c>
-      <c r="C46" s="40">
+      <c r="A46" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B46" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="C46" s="38">
         <f>N23</f>
         <v>1380000</v>
       </c>
-      <c r="D46" s="16" t="str">
+      <c r="D46" s="15" t="str">
         <f>IF(N23&gt;0,"Unfavorable","Favorable")</f>
         <v>Unfavorable</v>
       </c>
       <c r="E46" s="76" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F46" s="77"/>
       <c r="G46" s="77"/>
@@ -6610,22 +6725,22 @@
       <c r="N46" s="78"/>
     </row>
     <row r="47" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="39" t="s">
-        <v>16</v>
-      </c>
-      <c r="B47" s="42" t="s">
-        <v>13</v>
-      </c>
-      <c r="C47" s="41">
+      <c r="A47" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B47" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="C47" s="39">
         <f>M23</f>
         <v>300000</v>
       </c>
-      <c r="D47" s="16" t="str">
+      <c r="D47" s="15" t="str">
         <f>IF(M23&gt;0,"Unfavorable","Favorable")</f>
         <v>Unfavorable</v>
       </c>
       <c r="E47" s="76" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F47" s="77"/>
       <c r="G47" s="77"/>
@@ -6638,22 +6753,22 @@
       <c r="N47" s="78"/>
     </row>
     <row r="48" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="39" t="s">
-        <v>15</v>
-      </c>
-      <c r="B48" s="42" t="s">
-        <v>14</v>
-      </c>
-      <c r="C48" s="41">
+      <c r="A48" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="B48" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="C48" s="39">
         <f>N22</f>
         <v>465000</v>
       </c>
-      <c r="D48" s="16" t="str">
+      <c r="D48" s="15" t="str">
         <f>IF(N22&gt;0,"Unfavorable","Favorable")</f>
         <v>Unfavorable</v>
       </c>
       <c r="E48" s="76" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F48" s="77"/>
       <c r="G48" s="77"/>
@@ -6666,22 +6781,22 @@
       <c r="N48" s="78"/>
     </row>
     <row r="49" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="38" t="s">
-        <v>17</v>
-      </c>
-      <c r="B49" s="42" t="s">
-        <v>14</v>
-      </c>
-      <c r="C49" s="41">
+      <c r="A49" s="36" t="s">
+        <v>35</v>
+      </c>
+      <c r="B49" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="C49" s="39">
         <f>N24</f>
         <v>-610000</v>
       </c>
-      <c r="D49" s="16" t="str">
+      <c r="D49" s="15" t="str">
         <f>IF(N24&gt;0,"Unfavorable","Favorable")</f>
         <v>Favorable</v>
       </c>
       <c r="E49" s="76" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="F49" s="77"/>
       <c r="G49" s="77"/>
@@ -6694,22 +6809,22 @@
       <c r="N49" s="78"/>
     </row>
     <row r="50" spans="1:14" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="38" t="s">
-        <v>18</v>
-      </c>
-      <c r="B50" s="42" t="s">
-        <v>11</v>
-      </c>
-      <c r="C50" s="41">
+      <c r="A50" s="36" t="s">
+        <v>37</v>
+      </c>
+      <c r="B50" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="C50" s="39">
         <f>K25</f>
         <v>160000</v>
       </c>
-      <c r="D50" s="16" t="str">
+      <c r="D50" s="15" t="str">
         <f>IF(K25&gt;0,"Unfavorable","Favorable")</f>
         <v>Unfavorable</v>
       </c>
       <c r="E50" s="76" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F50" s="77"/>
       <c r="G50" s="77"/>
@@ -6722,19 +6837,21 @@
       <c r="N50" s="78"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A44:N44"/>
+    <mergeCell ref="A4:N4"/>
+    <mergeCell ref="A12:N12"/>
+    <mergeCell ref="A20:N20"/>
+    <mergeCell ref="A28:N28"/>
+    <mergeCell ref="A36:N36"/>
     <mergeCell ref="E50:N50"/>
     <mergeCell ref="E45:N45"/>
     <mergeCell ref="E46:N46"/>
     <mergeCell ref="E47:N47"/>
     <mergeCell ref="E48:N48"/>
     <mergeCell ref="E49:N49"/>
-    <mergeCell ref="A44:N44"/>
-    <mergeCell ref="A4:N4"/>
-    <mergeCell ref="A12:N12"/>
-    <mergeCell ref="A20:N20"/>
-    <mergeCell ref="A28:N28"/>
-    <mergeCell ref="A36:N36"/>
   </mergeCells>
   <conditionalFormatting sqref="B38:N42">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
@@ -6754,192 +6871,194 @@
   <dimension ref="A1:Y26"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" style="30" customWidth="1"/>
-    <col min="2" max="3" width="8.85546875" style="30"/>
-    <col min="4" max="4" width="8.85546875" style="30" customWidth="1"/>
-    <col min="5" max="5" width="3" style="30" customWidth="1"/>
-    <col min="6" max="6" width="8.85546875" style="30"/>
-    <col min="7" max="7" width="8.85546875" style="30" customWidth="1"/>
-    <col min="8" max="8" width="8.85546875" style="30"/>
-    <col min="9" max="9" width="3" style="30" customWidth="1"/>
-    <col min="10" max="12" width="8.85546875" style="30" customWidth="1"/>
-    <col min="13" max="13" width="3" style="30" customWidth="1"/>
-    <col min="14" max="16384" width="8.85546875" style="30"/>
+    <col min="1" max="1" width="10.5703125" style="28" customWidth="1"/>
+    <col min="2" max="3" width="8.85546875" style="28"/>
+    <col min="4" max="4" width="8.85546875" style="28" customWidth="1"/>
+    <col min="5" max="5" width="3" style="28" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="28"/>
+    <col min="7" max="7" width="8.85546875" style="28" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" style="28"/>
+    <col min="9" max="9" width="3" style="28" customWidth="1"/>
+    <col min="10" max="12" width="8.85546875" style="28" customWidth="1"/>
+    <col min="13" max="13" width="3" style="28" customWidth="1"/>
+    <col min="14" max="18" width="8.85546875" style="28"/>
+    <col min="19" max="19" width="10.28515625" style="28" bestFit="1" customWidth="1"/>
+    <col min="20" max="16384" width="8.85546875" style="28"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="22.5" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="7.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="29"/>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
+      <c r="A2" s="27"/>
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
     </row>
     <row r="3" spans="1:16" ht="13.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="45"/>
-      <c r="B3" s="88" t="s">
-        <v>50</v>
-      </c>
-      <c r="C3" s="88"/>
-      <c r="D3" s="88"/>
-      <c r="F3" s="88" t="s">
-        <v>49</v>
-      </c>
-      <c r="G3" s="88"/>
-      <c r="H3" s="88"/>
-      <c r="J3" s="89" t="s">
+      <c r="A3" s="43"/>
+      <c r="B3" s="93" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" s="93"/>
+      <c r="D3" s="93"/>
+      <c r="F3" s="93" t="s">
         <v>71</v>
       </c>
-      <c r="K3" s="90"/>
-      <c r="L3" s="91"/>
-      <c r="N3" s="89" t="s">
-        <v>22</v>
-      </c>
-      <c r="O3" s="90"/>
-      <c r="P3" s="91"/>
+      <c r="G3" s="93"/>
+      <c r="H3" s="93"/>
+      <c r="J3" s="94" t="s">
+        <v>72</v>
+      </c>
+      <c r="K3" s="95"/>
+      <c r="L3" s="96"/>
+      <c r="N3" s="94" t="s">
+        <v>63</v>
+      </c>
+      <c r="O3" s="95"/>
+      <c r="P3" s="96"/>
     </row>
     <row r="4" spans="1:16" ht="13.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="45"/>
-      <c r="B4" s="88"/>
-      <c r="C4" s="88"/>
-      <c r="D4" s="88"/>
-      <c r="F4" s="88"/>
-      <c r="G4" s="88"/>
-      <c r="H4" s="88"/>
-      <c r="J4" s="92"/>
-      <c r="K4" s="93"/>
-      <c r="L4" s="94"/>
-      <c r="N4" s="92"/>
-      <c r="O4" s="93"/>
-      <c r="P4" s="94"/>
+      <c r="A4" s="43"/>
+      <c r="B4" s="93"/>
+      <c r="C4" s="93"/>
+      <c r="D4" s="93"/>
+      <c r="F4" s="93"/>
+      <c r="G4" s="93"/>
+      <c r="H4" s="93"/>
+      <c r="J4" s="97"/>
+      <c r="K4" s="98"/>
+      <c r="L4" s="99"/>
+      <c r="N4" s="100"/>
+      <c r="O4" s="101"/>
+      <c r="P4" s="102"/>
     </row>
     <row r="5" spans="1:16" ht="13.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="45"/>
-      <c r="B5" s="80">
+      <c r="A5" s="43"/>
+      <c r="B5" s="86">
         <f>'Budget vs Actual'!N10</f>
         <v>47950000</v>
       </c>
-      <c r="C5" s="81"/>
-      <c r="D5" s="82"/>
-      <c r="F5" s="80">
+      <c r="C5" s="87"/>
+      <c r="D5" s="88"/>
+      <c r="F5" s="86">
         <f>'Budget vs Actual'!N18</f>
         <v>49361000</v>
       </c>
-      <c r="G5" s="81"/>
-      <c r="H5" s="82"/>
-      <c r="J5" s="86">
+      <c r="G5" s="87"/>
+      <c r="H5" s="88"/>
+      <c r="J5" s="92">
         <f>'Budget vs Actual'!N26</f>
         <v>1411000</v>
       </c>
-      <c r="K5" s="86"/>
-      <c r="L5" s="86"/>
-      <c r="N5" s="87" t="str">
+      <c r="K5" s="92"/>
+      <c r="L5" s="92"/>
+      <c r="N5" s="103" t="str">
         <f>IF('Budget vs Actual'!N26&gt;0,"Unfavorable","Favorable")</f>
         <v>Unfavorable</v>
       </c>
-      <c r="O5" s="87"/>
-      <c r="P5" s="87"/>
+      <c r="O5" s="104"/>
+      <c r="P5" s="105"/>
     </row>
     <row r="6" spans="1:16" ht="13.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="45"/>
-      <c r="B6" s="80"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="82"/>
-      <c r="F6" s="80"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="82"/>
-      <c r="J6" s="86"/>
-      <c r="K6" s="86"/>
-      <c r="L6" s="86"/>
-      <c r="N6" s="87"/>
-      <c r="O6" s="87"/>
-      <c r="P6" s="87"/>
+      <c r="A6" s="43"/>
+      <c r="B6" s="86"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="88"/>
+      <c r="F6" s="86"/>
+      <c r="G6" s="87"/>
+      <c r="H6" s="88"/>
+      <c r="J6" s="92"/>
+      <c r="K6" s="92"/>
+      <c r="L6" s="92"/>
+      <c r="N6" s="103"/>
+      <c r="O6" s="104"/>
+      <c r="P6" s="105"/>
     </row>
     <row r="7" spans="1:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="46"/>
-      <c r="B7" s="83"/>
-      <c r="C7" s="84"/>
-      <c r="D7" s="85"/>
-      <c r="F7" s="83"/>
-      <c r="G7" s="84"/>
-      <c r="H7" s="85"/>
-      <c r="J7" s="86"/>
-      <c r="K7" s="86"/>
-      <c r="L7" s="86"/>
-      <c r="N7" s="87"/>
-      <c r="O7" s="87"/>
-      <c r="P7" s="87"/>
+      <c r="A7" s="44"/>
+      <c r="B7" s="89"/>
+      <c r="C7" s="90"/>
+      <c r="D7" s="91"/>
+      <c r="F7" s="89"/>
+      <c r="G7" s="90"/>
+      <c r="H7" s="91"/>
+      <c r="J7" s="92"/>
+      <c r="K7" s="92"/>
+      <c r="L7" s="92"/>
+      <c r="N7" s="103"/>
+      <c r="O7" s="104"/>
+      <c r="P7" s="105"/>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="O9" s="30" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L10" s="30" t="s">
-        <v>50</v>
-      </c>
-      <c r="M10" s="33">
+      <c r="O9" s="28" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="L10" s="28" t="s">
+        <v>70</v>
+      </c>
+      <c r="M10" s="31">
         <f>'Budget vs Actual'!N10</f>
         <v>47950000</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C11" s="30" t="s">
-        <v>55</v>
-      </c>
-      <c r="L11" s="30" t="s">
-        <v>51</v>
-      </c>
-      <c r="M11" s="33">
+    <row r="11" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="28" t="s">
+        <v>73</v>
+      </c>
+      <c r="L11" s="28" t="s">
+        <v>74</v>
+      </c>
+      <c r="M11" s="31">
         <f>'Budget vs Actual'!N22</f>
         <v>465000</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="C12" s="30" t="s">
-        <v>56</v>
-      </c>
-      <c r="L12" s="34" t="s">
-        <v>52</v>
-      </c>
-      <c r="M12" s="33">
+    <row r="12" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C12" s="28" t="s">
+        <v>75</v>
+      </c>
+      <c r="L12" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="M12" s="31">
         <f>'Budget vs Actual'!N23</f>
         <v>1380000</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L13" s="30" t="s">
-        <v>53</v>
-      </c>
-      <c r="M13" s="33">
+      <c r="L13" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="M13" s="31">
         <f>'Budget vs Actual'!N24</f>
         <v>-610000</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L14" s="30" t="s">
-        <v>54</v>
-      </c>
-      <c r="M14" s="33">
+      <c r="L14" s="28" t="s">
+        <v>78</v>
+      </c>
+      <c r="M14" s="31">
         <f>'Budget vs Actual'!N25</f>
         <v>176000</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="L15" s="30" t="s">
-        <v>49</v>
-      </c>
-      <c r="M15" s="33">
+      <c r="L15" s="28" t="s">
+        <v>71</v>
+      </c>
+      <c r="M15" s="31">
         <f>'Budget vs Actual'!N18</f>
         <v>49361000</v>
       </c>
     </row>
     <row r="26" spans="25:25" x14ac:dyDescent="0.25">
-      <c r="Y26" s="31"/>
+      <c r="Y26" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -6958,7 +7077,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="1" id="{14B302FB-6033-4692-B48E-293C85487313}">
+          <x14:cfRule type="expression" priority="3" id="{14B302FB-6033-4692-B48E-293C85487313}">
             <xm:f>'Budget vs Actual'!$N$26&lt;0</xm:f>
             <x14:dxf>
               <fill>
@@ -6968,7 +7087,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <x14:cfRule type="expression" priority="4" id="{D77AA8C3-AA75-4A94-95A5-CF4AFEDEC850}">
+          <x14:cfRule type="expression" priority="6" id="{D77AA8C3-AA75-4A94-95A5-CF4AFEDEC850}">
             <xm:f>'Budget vs Actual'!$N$26&gt;0</xm:f>
             <x14:dxf>
               <fill>

</xml_diff>